<commit_message>
Rebuild 21.08.2026 weekly reports from updated TAZ
Regenerate Utair, Belavia and Aeroflot status files after delivery
dates were filled in the source TAZ export.

Co-authored-by: alexanderp-cell <alexanderp-cell@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/Utair статус 21.08.2026.xlsx
+++ b/output/Utair статус 21.08.2026.xlsx
@@ -788,7 +788,7 @@
         <v>3279161</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>485587.6199999995</v>
+        <v>485587.62</v>
       </c>
       <c r="G10" s="12" t="n">
         <v>2029235</v>
@@ -5036,8 +5036,8 @@
       <c r="V11" s="30" t="n">
         <v>46185</v>
       </c>
-      <c r="W11" s="27" t="n">
-        <v/>
+      <c r="W11" s="30" t="n">
+        <v>46246</v>
       </c>
       <c r="X11" s="27" t="inlineStr">
         <is>
@@ -5543,8 +5543,8 @@
       <c r="V13" s="30" t="n">
         <v>46197</v>
       </c>
-      <c r="W13" s="27" t="n">
-        <v/>
+      <c r="W13" s="30" t="n">
+        <v>46246</v>
       </c>
       <c r="X13" s="27" t="inlineStr">
         <is>
@@ -6806,8 +6806,8 @@
       <c r="V18" s="33" t="n">
         <v>46207</v>
       </c>
-      <c r="W18" s="19" t="n">
-        <v/>
+      <c r="W18" s="33" t="n">
+        <v>46226</v>
       </c>
       <c r="X18" s="19" t="inlineStr">
         <is>
@@ -7064,8 +7064,8 @@
       <c r="V19" s="30" t="n">
         <v>46217.46131</v>
       </c>
-      <c r="W19" s="27" t="n">
-        <v/>
+      <c r="W19" s="30" t="n">
+        <v>46246</v>
       </c>
       <c r="X19" s="27" t="inlineStr">
         <is>
@@ -7815,8 +7815,8 @@
       <c r="V22" s="33" t="n">
         <v>46225</v>
       </c>
-      <c r="W22" s="19" t="n">
-        <v/>
+      <c r="W22" s="33" t="n">
+        <v>46226</v>
       </c>
       <c r="X22" s="19" t="inlineStr">
         <is>
@@ -8071,8 +8071,8 @@
       <c r="V23" s="30" t="n">
         <v>46225</v>
       </c>
-      <c r="W23" s="27" t="n">
-        <v/>
+      <c r="W23" s="30" t="n">
+        <v>46226</v>
       </c>
       <c r="X23" s="27" t="inlineStr">
         <is>
@@ -8327,8 +8327,8 @@
       <c r="V24" s="33" t="n">
         <v>46227</v>
       </c>
-      <c r="W24" s="19" t="n">
-        <v/>
+      <c r="W24" s="33" t="n">
+        <v>46247</v>
       </c>
       <c r="X24" s="19" t="inlineStr">
         <is>
@@ -9327,8 +9327,8 @@
       <c r="V28" s="33" t="n">
         <v>46232</v>
       </c>
-      <c r="W28" s="19" t="n">
-        <v/>
+      <c r="W28" s="33" t="n">
+        <v>46246</v>
       </c>
       <c r="X28" s="19" t="inlineStr">
         <is>
@@ -9581,8 +9581,8 @@
       <c r="V29" s="30" t="n">
         <v>46232</v>
       </c>
-      <c r="W29" s="27" t="n">
-        <v/>
+      <c r="W29" s="30" t="n">
+        <v>46242</v>
       </c>
       <c r="X29" s="27" t="inlineStr">
         <is>
@@ -9828,8 +9828,8 @@
       <c r="V30" s="33" t="n">
         <v>46232</v>
       </c>
-      <c r="W30" s="19" t="n">
-        <v/>
+      <c r="W30" s="33" t="n">
+        <v>46246</v>
       </c>
       <c r="X30" s="19" t="inlineStr">
         <is>
@@ -10082,8 +10082,8 @@
       <c r="V31" s="30" t="n">
         <v>46239</v>
       </c>
-      <c r="W31" s="27" t="n">
-        <v/>
+      <c r="W31" s="30" t="n">
+        <v>46246</v>
       </c>
       <c r="X31" s="27" t="inlineStr">
         <is>
@@ -10575,8 +10575,8 @@
       <c r="V33" s="30" t="n">
         <v>46242</v>
       </c>
-      <c r="W33" s="27" t="n">
-        <v/>
+      <c r="W33" s="30" t="n">
+        <v>46246</v>
       </c>
       <c r="X33" s="27" t="inlineStr">
         <is>
@@ -11299,8 +11299,8 @@
       <c r="V36" s="33" t="n">
         <v>46246</v>
       </c>
-      <c r="W36" s="19" t="n">
-        <v/>
+      <c r="W36" s="33" t="n">
+        <v>46246</v>
       </c>
       <c r="X36" s="19" t="inlineStr">
         <is>
@@ -11553,8 +11553,8 @@
       <c r="V37" s="30" t="n">
         <v>46247</v>
       </c>
-      <c r="W37" s="27" t="n">
-        <v/>
+      <c r="W37" s="30" t="n">
+        <v>46246</v>
       </c>
       <c r="X37" s="27" t="inlineStr">
         <is>
@@ -11808,8 +11808,8 @@
       <c r="V38" s="33" t="n">
         <v>46229</v>
       </c>
-      <c r="W38" s="19" t="n">
-        <v/>
+      <c r="W38" s="33" t="n">
+        <v>46242</v>
       </c>
       <c r="X38" s="19" t="inlineStr">
         <is>
@@ -12058,8 +12058,8 @@
       <c r="V39" s="30" t="n">
         <v>46242</v>
       </c>
-      <c r="W39" s="27" t="n">
-        <v/>
+      <c r="W39" s="30" t="n">
+        <v>46247</v>
       </c>
       <c r="X39" s="27" t="inlineStr">
         <is>
@@ -12304,8 +12304,8 @@
       <c r="V40" s="33" t="n">
         <v>46248</v>
       </c>
-      <c r="W40" s="19" t="n">
-        <v/>
+      <c r="W40" s="33" t="n">
+        <v>46246</v>
       </c>
       <c r="X40" s="19" t="inlineStr">
         <is>
@@ -12558,8 +12558,8 @@
       <c r="V41" s="30" t="n">
         <v>46250</v>
       </c>
-      <c r="W41" s="27" t="n">
-        <v/>
+      <c r="W41" s="30" t="n">
+        <v>46246</v>
       </c>
       <c r="X41" s="27" t="inlineStr">
         <is>
@@ -12812,8 +12812,8 @@
       <c r="V42" s="33" t="n">
         <v>46248</v>
       </c>
-      <c r="W42" s="19" t="n">
-        <v/>
+      <c r="W42" s="33" t="n">
+        <v>46246</v>
       </c>
       <c r="X42" s="19" t="inlineStr">
         <is>
@@ -13066,8 +13066,8 @@
       <c r="V43" s="30" t="n">
         <v>46265</v>
       </c>
-      <c r="W43" s="27" t="n">
-        <v/>
+      <c r="W43" s="30" t="n">
+        <v>46246</v>
       </c>
       <c r="X43" s="27" t="inlineStr">
         <is>
@@ -13320,8 +13320,8 @@
       <c r="V44" s="33" t="n">
         <v>46256</v>
       </c>
-      <c r="W44" s="19" t="n">
-        <v/>
+      <c r="W44" s="33" t="n">
+        <v>46247</v>
       </c>
       <c r="X44" s="19" t="inlineStr">
         <is>
@@ -19169,7 +19169,7 @@
       </c>
       <c r="BB22" s="19" t="inlineStr">
         <is>
-          <t>UNCONFIRMED YET</t>
+          <t>HA WHS</t>
         </is>
       </c>
       <c r="BC22" s="19" t="n">
@@ -19181,8 +19181,10 @@
       <c r="BE22" s="19" t="n">
         <v/>
       </c>
-      <c r="BF22" s="19" t="n">
-        <v/>
+      <c r="BF22" s="19" t="inlineStr">
+        <is>
+          <t>Др</t>
+        </is>
       </c>
       <c r="BG22" s="19" t="n">
         <v/>
@@ -24763,7 +24765,7 @@
       </c>
       <c r="BB45" s="27" t="inlineStr">
         <is>
-          <t>UNCONFIRMED YET</t>
+          <t>HA WHS</t>
         </is>
       </c>
       <c r="BC45" s="27" t="n">
@@ -24775,8 +24777,10 @@
       <c r="BE45" s="27" t="n">
         <v/>
       </c>
-      <c r="BF45" s="27" t="n">
-        <v/>
+      <c r="BF45" s="27" t="inlineStr">
+        <is>
+          <t>Др</t>
+        </is>
       </c>
       <c r="BG45" s="27" t="n">
         <v/>

</xml_diff>